<commit_message>
Update the cohort upload template (#319)
With the new column `CHILD_CLINICALLY_AT_RISK_FOR_FLU`. This matches
the code changes in production:
https://github.com/NHSDigital/manage-vaccinations-in-schools/pull/7862
</commit_message>
<xml_diff>
--- a/app/files/cohort-upload-template.xlsx
+++ b/app/files/cohort-upload-template.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28712"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FEC1538-FFB1-4056-BB0D-6C73AD442E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alistair/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA44E12-863C-7744-8B46-0C61BD9C3D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="complete template" sheetId="2" r:id="rId1"/>
@@ -31,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>CHILD_SCHOOL_URN</t>
   </si>
@@ -201,12 +206,18 @@
   <si>
     <t>Optional: Email address </t>
   </si>
+  <si>
+    <t>CHILD_CLINICALLY_AT_RISK_FOR_FLU</t>
+  </si>
+  <si>
+    <t>Optional, must be one of: true, yes, 1 or y for yes, or false, no, 0 or n for no. If absent or blank, defaults to no.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,6 +254,18 @@
       <sz val="10"/>
       <color rgb="FF0F0F0F"/>
       <name val="Helvetica"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0F0F0F"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0F0F0F"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -286,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -316,6 +339,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -652,32 +681,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE0FF976-7385-4EFB-92FB-A6D5246D9732}">
-  <dimension ref="A1:W2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:X2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" customWidth="1"/>
-    <col min="2" max="2" width="25.28515625" customWidth="1"/>
-    <col min="3" max="5" width="23.85546875" customWidth="1"/>
-    <col min="6" max="6" width="28.5703125" customWidth="1"/>
-    <col min="7" max="8" width="30.85546875" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" customWidth="1"/>
-    <col min="10" max="10" width="32" customWidth="1"/>
-    <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="23.28515625" customWidth="1"/>
-    <col min="13" max="13" width="27.140625" customWidth="1"/>
-    <col min="14" max="15" width="29.5703125" customWidth="1"/>
-    <col min="16" max="16" width="31.28515625" customWidth="1"/>
-    <col min="17" max="17" width="22.5703125" customWidth="1"/>
-    <col min="18" max="18" width="21.5703125" customWidth="1"/>
-    <col min="19" max="19" width="31.140625" customWidth="1"/>
-    <col min="20" max="20" width="31.5703125" customWidth="1"/>
-    <col min="21" max="21" width="31.42578125" customWidth="1"/>
-    <col min="22" max="22" width="26.7109375" customWidth="1"/>
-    <col min="23" max="23" width="23.5703125" customWidth="1"/>
-    <col min="24" max="24" width="28.42578125" customWidth="1"/>
+    <col min="1" max="1" width="23.1640625" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="21.5" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22.1640625" customWidth="1"/>
+    <col min="6" max="6" width="25.33203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" customWidth="1"/>
+    <col min="10" max="10" width="27.5" customWidth="1"/>
+    <col min="11" max="11" width="27.6640625" customWidth="1"/>
+    <col min="12" max="12" width="15.6640625" customWidth="1"/>
+    <col min="13" max="13" width="20.1640625" customWidth="1"/>
+    <col min="14" max="14" width="23.6640625" customWidth="1"/>
+    <col min="15" max="15" width="41.5" customWidth="1"/>
+    <col min="16" max="16" width="19.1640625" customWidth="1"/>
+    <col min="17" max="17" width="28.1640625" customWidth="1"/>
+    <col min="18" max="18" width="20.6640625" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="18.83203125" customWidth="1"/>
+    <col min="21" max="21" width="28" customWidth="1"/>
+    <col min="22" max="22" width="21" customWidth="1"/>
+    <col min="23" max="23" width="19.6640625" customWidth="1"/>
+    <col min="24" max="24" width="23.5" customWidth="1"/>
+    <col min="25" max="25" width="28.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="1" customFormat="1" ht="36">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -720,33 +754,36 @@
       <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
     </row>
-    <row r="2" spans="1:23" s="2" customFormat="1" ht="51" customHeight="1">
+    <row r="2" spans="1:24" s="2" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>22</v>
       </c>
@@ -789,31 +826,34 @@
       <c r="N2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -821,6 +861,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <DocType xmlns="80d05917-893e-4a06-bb39-47099b578ffd" xsi:nil="true"/>
@@ -837,15 +886,6 @@
     <TaxCatchAll xmlns="754dda3c-967d-4b24-9bc2-1cc61ceab4bc" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1141,13 +1181,41 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C876B08D-714B-4BF4-B883-950097757B90}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AA4DC00-880E-449F-B2E3-25A12598E9D3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AA4DC00-880E-449F-B2E3-25A12598E9D3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C876B08D-714B-4BF4-B883-950097757B90}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="80d05917-893e-4a06-bb39-47099b578ffd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="754dda3c-967d-4b24-9bc2-1cc61ceab4bc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B9C5003-FBBA-4869-9A5A-77A53BE546C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B9C5003-FBBA-4869-9A5A-77A53BE546C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="80d05917-893e-4a06-bb39-47099b578ffd"/>
+    <ds:schemaRef ds:uri="754dda3c-967d-4b24-9bc2-1cc61ceab4bc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>